<commit_message>
EXCEL add main 2
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\gittest_20260323\git-branching\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4B9D38C4-AFBD-4AF1-B0F7-7C09918C84F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55AEAD4F-9F69-48CD-B353-A99DF0440172}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3936" yWindow="3276" windowWidth="17280" windowHeight="8964" xr2:uid="{584B7A33-545A-4F0A-93B5-3753C02A12B8}"/>
   </bookViews>
@@ -22,6 +22,23 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+  <si>
+    <t>aaaaaaaaaaaaaaaaa</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>bbbbbbbbbbbbbbbb</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ccccccccccccccccc</t>
+    <phoneticPr fontId="1"/>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -383,9 +400,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A6E11FA-BBB1-43B7-8C0D-71D624FBE4DA}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>